<commit_message>
item kosten angepasst, rüstung nun flat, bildschirm scaling fix
</commit_message>
<xml_diff>
--- a/items_list.xlsx
+++ b/items_list.xlsx
@@ -497,13 +497,13 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -541,10 +541,10 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -582,10 +582,10 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -661,13 +661,13 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -702,13 +702,13 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -743,13 +743,13 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -784,13 +784,13 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -825,13 +825,13 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -866,13 +866,13 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -910,10 +910,10 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I12" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -951,10 +951,10 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I13" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -992,10 +992,10 @@
         <v>1</v>
       </c>
       <c r="H14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I14" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -1033,10 +1033,10 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I15" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -1077,7 +1077,7 @@
         <v>4</v>
       </c>
       <c r="I16" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -1115,10 +1115,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I17" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -1156,10 +1156,10 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="I18" t="n">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -1200,7 +1200,7 @@
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -1241,7 +1241,7 @@
         <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -1282,7 +1282,7 @@
         <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
@@ -1317,13 +1317,13 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -1358,13 +1358,13 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -1402,10 +1402,10 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I24" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="I25" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
@@ -1484,10 +1484,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I26" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
@@ -1528,7 +1528,7 @@
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -1569,7 +1569,7 @@
         <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="G29" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -1645,13 +1645,13 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H30" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I30" t="n">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
@@ -1686,13 +1686,13 @@
         </is>
       </c>
       <c r="G31" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="H31" t="n">
         <v>0</v>
       </c>
       <c r="I31" t="n">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
@@ -1727,13 +1727,13 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
@@ -1768,13 +1768,13 @@
         </is>
       </c>
       <c r="G33" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
@@ -1809,13 +1809,13 @@
         </is>
       </c>
       <c r="G34" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H34" t="n">
         <v>0</v>
       </c>
       <c r="I34" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
@@ -1850,13 +1850,13 @@
         </is>
       </c>
       <c r="G35" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H35" t="n">
         <v>0</v>
       </c>
       <c r="I35" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
@@ -1891,13 +1891,13 @@
         </is>
       </c>
       <c r="G36" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="H36" t="n">
         <v>0</v>
       </c>
       <c r="I36" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
@@ -1932,13 +1932,13 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H37" t="n">
         <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
@@ -1973,13 +1973,13 @@
         </is>
       </c>
       <c r="G38" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I38" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
@@ -2017,10 +2017,10 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I39" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
@@ -2058,10 +2058,10 @@
         <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I40" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
@@ -2102,7 +2102,7 @@
         <v>4</v>
       </c>
       <c r="I41" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
@@ -2140,10 +2140,10 @@
         <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I42" t="n">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
@@ -2181,10 +2181,10 @@
         <v>0</v>
       </c>
       <c r="H43" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="I43" t="n">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>
@@ -2219,13 +2219,13 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H44" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I44" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
@@ -2266,7 +2266,7 @@
         <v>3</v>
       </c>
       <c r="I45" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="J45" t="inlineStr">
         <is>
@@ -2307,7 +2307,7 @@
         <v>0</v>
       </c>
       <c r="I46" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
@@ -2348,7 +2348,7 @@
         <v>0</v>
       </c>
       <c r="I47" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
@@ -2389,7 +2389,7 @@
         <v>0</v>
       </c>
       <c r="I48" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
@@ -2430,7 +2430,7 @@
         <v>0</v>
       </c>
       <c r="I49" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="J49" t="inlineStr">
         <is>
@@ -2468,10 +2468,10 @@
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I50" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="J50" t="inlineStr">
         <is>
@@ -2506,13 +2506,13 @@
         </is>
       </c>
       <c r="G51" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="H51" t="n">
         <v>0</v>
       </c>
       <c r="I51" t="n">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="J51" t="inlineStr">
         <is>
@@ -2547,13 +2547,13 @@
         </is>
       </c>
       <c r="G52" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H52" t="n">
         <v>0</v>
       </c>
       <c r="I52" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
@@ -2588,13 +2588,13 @@
         </is>
       </c>
       <c r="G53" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="H53" t="n">
         <v>0</v>
       </c>
       <c r="I53" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="J53" t="inlineStr">
         <is>
@@ -2635,7 +2635,7 @@
         <v>1</v>
       </c>
       <c r="I54" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J54" t="inlineStr">
         <is>
@@ -2676,7 +2676,7 @@
         <v>4</v>
       </c>
       <c r="I55" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="J55" t="inlineStr">
         <is>
@@ -2711,13 +2711,13 @@
         </is>
       </c>
       <c r="G56" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H56" t="n">
         <v>5</v>
       </c>
       <c r="I56" t="n">
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="J56" t="inlineStr">
         <is>
@@ -2755,10 +2755,10 @@
         <v>0</v>
       </c>
       <c r="H57" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="I57" t="n">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="J57" t="inlineStr">
         <is>
@@ -2793,13 +2793,13 @@
         </is>
       </c>
       <c r="G58" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="H58" t="n">
         <v>0</v>
       </c>
       <c r="I58" t="n">
-        <v>75</v>
+        <v>10</v>
       </c>
       <c r="J58" t="inlineStr">
         <is>
@@ -2834,13 +2834,13 @@
         </is>
       </c>
       <c r="G59" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H59" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I59" t="n">
-        <v>50</v>
+        <v>9</v>
       </c>
       <c r="J59" t="inlineStr">
         <is>
@@ -2881,7 +2881,7 @@
         <v>0</v>
       </c>
       <c r="I60" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="J60" t="inlineStr">
         <is>
@@ -2922,7 +2922,7 @@
         <v>0</v>
       </c>
       <c r="I61" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="J61" t="inlineStr">
         <is>

</xml_diff>